<commit_message>
Pendientes del tomo I: decisiones al Excel, índice de créditos en el tomo II
</commit_message>
<xml_diff>
--- a/investigacion/errores_tomo1_2026-10-22/protocolo_vs_libro.xlsx
+++ b/investigacion/errores_tomo1_2026-10-22/protocolo_vs_libro.xlsx
@@ -503,7 +503,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Hoja "Decide tú": lo único que hay que decidir. El libro hoy NO sigue al protocolo en estas prácticas. En la última columna elige Protocolo (el libro vuelve al protocolo y lo otro queda como observación), Dejar como está, o Conversarlo.</t>
+          <t>Hoja "Decide tú": lo único que hay que decidir. El libro hoy NO sigue al protocolo en estas prácticas, más dos decisiones tuyas del tomo I (restricciones después de la maniobra en H19 y el símbolo del LDL en H3). En la última columna elige Protocolo (el libro vuelve al protocolo y lo otro queda como observación), Dejar como está, o Conversarlo.</t>
         </is>
       </c>
     </row>
@@ -552,14 +552,14 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Decide tú: 0 resueltas, 26 pendientes, 0 ya no aplican (26 filas)</t>
+          <t xml:space="preserve">  Decide tú: 0 resueltas, 28 pendientes, 0 ya no aplican (28 filas)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ya sigue al protocolo: 67 resueltas, 0 pendientes, 0 ya no aplican (67 filas)</t>
+          <t xml:space="preserve">  Ya sigue al protocolo: 66 resueltas, 0 pendientes, 0 ya no aplican (66 filas)</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2046,9 +2046,115 @@
       </c>
       <c r="K27" s="5" t="inlineStr"/>
     </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>H19</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Indicaciones después de la maniobra</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Qué se le indica al paciente para dormir y moverse después de la maniobra de reposición.</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Dormir semisentado 2 noches, sin movimientos bruscos.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Pone lo del protocolo; en el recuadro, la AAO-HNS 2017 recomienda con fuerza NO indicar restricciones (grado A).</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>AAO-HNS 2017 (Bhattacharyya)</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Si se deja: nada. Si se quita: el paso de H19 y el recuadro.</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="n"/>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>nuevo</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>LDL: qué símbolo y si se une</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Cómo se dibuja el umbral de molestia en el audiograma.</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>No define símbolo para el LDL ni si se une (solo líneas de aérea y ósea, colores y flecha).</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Triángulo relleno hacia abajo, unido con guiones. Pedido pendiente (2026-10-16): mostrar todas las convenciones (triángulo chileno, └ ┘ de la BSA, "m" en España, "U" en inglés) y decir que unir o no es elección.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>investigacion/simbolo_ldl.md (BSA 2022 lo deja sin unir; ninguna norma pide unirlo)</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Lámina de símbolos de H3, el texto y todas las figuras con LDL (motor).</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="K2 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28:K29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Protocolo,Dejar como está,Conversarlo"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2062,7 +2168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3044,7 +3150,7 @@
     <row r="24" ht="44.5" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -3054,22 +3160,22 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Indicaciones después de la maniobra</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Qué se indica al paciente para el reposo después de la maniobra.</t>
+          <t>Cuándo se controla al paciente después de la maniobra.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>dormir semisentado 2 noches, sin movimientos bruscos</t>
+          <t>a los 7 días</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; en el recuadro, la AAO-HNS recomienda con fuerza NO indicar restricciones (grado A)</t>
+          <t>el protocolo; en el recuadro, reevaluar dentro del mes</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -3086,7 +3192,7 @@
     <row r="25" ht="31" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>hoy</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -3096,27 +3202,27 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Giro supino (supine roll)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Cuándo se controla al paciente después de la maniobra.</t>
+          <t>Cuánto se observa el nistagmo en cada lado.</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>a los 7 días</t>
+          <t>30 segundos por lado.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; en el recuadro, reevaluar dentro del mes</t>
+          <t>AAO-HNS: hasta que el nistagmo cese (el apogeotrópico puede durar más de 1 min).</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Antes (regla del autor, 2026-10-16)</t>
+          <t>Hoy (2026-10-22)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -3128,37 +3234,37 @@
     <row r="26" ht="31" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>hoy</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>H19</t>
+          <t>H20</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Giro supino (supine roll)</t>
+          <t>Ejercicios oculomotores con la cabeza quieta</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Cuánto se observa el nistagmo en cada lado.</t>
+          <t>Ejercicios de ojos con la cabeza quieta en la rehabilitación.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>30 segundos por lado.</t>
+          <t>"estimulan los núcleos vestibulares"</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>AAO-HNS: hasta que el nistagmo cese (el apogeotrópico puede durar más de 1 min).</t>
+          <t>se mantienen; recuadro: la guía APTA recomienda (evidencia fuerte) no ofrecerlos como estabilización de la mirada</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Hoy (2026-10-22)</t>
+          <t>Antes (regla del autor, 2026-10-16)</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -3170,7 +3276,7 @@
     <row r="27" ht="44.5" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -3180,22 +3286,22 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Ejercicios oculomotores con la cabeza quieta</t>
+          <t>Agudeza visual dinámica</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Ejercicios de ojos con la cabeza quieta en la rehabilitación.</t>
+          <t>A qué velocidad se mueve la cabeza en la prueba de visión dinámica.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>"estimulan los núcleos vestibulares"</t>
+          <t>a 3 Hz</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>se mantienen; recuadro: la guía APTA recomienda (evidencia fuerte) no ofrecerlos como estabilización de la mirada</t>
+          <t>el protocolo; recuadro con la versión clínica a 2 Hz</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -3212,7 +3318,7 @@
     <row r="28" ht="31" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>88</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -3222,22 +3328,22 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Agudeza visual dinámica</t>
+          <t>Dosis del programa</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>A qué velocidad se mueve la cabeza en la prueba de visión dinámica.</t>
+          <t>Cuántas semanas y sesiones dura el programa de rehabilitación.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>a 3 Hz</t>
+          <t>3 a 6 semanas, una sesión semanal, sin dosis en casa</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro con la versión clínica a 2 Hz</t>
+          <t>el protocolo + tabla con los mínimos diarios y las semanas de la guía</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -3254,32 +3360,32 @@
     <row r="29" ht="31" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>91</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>H20</t>
+          <t>H21</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Dosis del programa</t>
+          <t>Ajuste del audífono</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Cuántas semanas y sesiones dura el programa de rehabilitación.</t>
+          <t>Cómo se regula el audífono en la consulta.</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>3 a 6 semanas, una sesión semanal, sin dosis en casa</t>
+          <t>por comodidad ("¿más o menos fuerza?")</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>el protocolo + tabla con los mínimos diarios y las semanas de la guía</t>
+          <t>el protocolo; recuadro: objetivo prescriptivo y medición en oído real</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -3296,7 +3402,7 @@
     <row r="30" ht="31" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>92</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -3306,22 +3412,22 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Ajuste del audífono</t>
+          <t>Molestia</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Cómo se regula el audífono en la consulta.</t>
+          <t>Cómo se mide la molestia por ruido con el audífono.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>por comodidad ("¿más o menos fuerza?")</t>
+          <t>grito o ruido cerca del oído</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: objetivo prescriptivo y medición en oído real</t>
+          <t>el protocolo; lo medible es el LDL con estímulo calibrado (→ H5)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -3338,7 +3444,7 @@
     <row r="31" ht="31" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>93</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -3348,22 +3454,22 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Molestia</t>
+          <t>Palabras</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Cómo se mide la molestia por ruido con el audífono.</t>
+          <t>Qué palabras se usan para comparar con y sin audífono.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>grito o ruido cerca del oído</t>
+          <t>voz viva sin nivel</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; lo medible es el LDL con estímulo calibrado (→ H5)</t>
+          <t>el protocolo; recuadro: material grabado al mismo nivel con y sin audífono</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -3380,32 +3486,32 @@
     <row r="32" ht="31" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>96</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>H21</t>
+          <t>H22</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Palabras</t>
+          <t>Funciones adaptativas en la medición</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Qué palabras se usan para comparar con y sin audífono.</t>
+          <t>Si se apagan las funciones inteligentes al medir el audífono.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>voz viva sin nivel</t>
+          <t>no pide desactivarlas</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: material grabado al mismo nivel con y sin audífono</t>
+          <t>El protocolo mide con el programa habitual del usuario; el recuadro dice que la norma ANSI S3.22 pide apagar las funciones adaptativas y anotar lo activo.</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -3422,7 +3528,7 @@
     <row r="33" ht="58" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>97</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -3432,22 +3538,22 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Funciones adaptativas en la medición</t>
+          <t>Conclusión "audibilidad buena/regular/mala"</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Si se apagan las funciones inteligentes al medir el audífono.</t>
+          <t>Cómo se concluye si el audífono da buena audibilidad.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>no pide desactivarlas</t>
+          <t>desde la medición en acoplador</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>El protocolo mide con el programa habitual del usuario; el recuadro dice que la norma ANSI S3.22 pide apagar las funciones adaptativas y anotar lo activo.</t>
+          <t>el protocolo; recuadro: la norma es de control de calidad, no de verificación</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -3464,7 +3570,7 @@
     <row r="34" ht="31" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>hoy</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -3474,27 +3580,27 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Conclusión "audibilidad buena/regular/mala"</t>
+          <t>Tubo al acoplador del audífono</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Cómo se concluye si el audífono da buena audibilidad.</t>
+          <t>Cómo se une el audífono al acoplador de 2 cm³ para medirlo.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>desde la medición en acoplador</t>
+          <t>Tubo flexible de unos 1,5 cm.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: la norma es de control de calidad, no de verificación</t>
+          <t>Norma (Cole y Chasin): 25 mm entre el gancho y el molde; parte lo pone el usuario.</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Antes (regla del autor, 2026-10-16)</t>
+          <t>Hoy (2026-10-22) · ver también N.º 98</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -3506,37 +3612,37 @@
     <row r="35" ht="31" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>hoy</t>
+          <t>102</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>H22</t>
+          <t>H25</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Tubo al acoplador del audífono</t>
+          <t>Aclimatación</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Cómo se une el audífono al acoplador de 2 cm³ para medirlo.</t>
+          <t>Cuántos minutos espera el paciente antes de mirar o medir la nariz.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Tubo flexible de unos 1,5 cm.</t>
+          <t>15 min en la preparación; "desde los 10 min" en la rinoscopía</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Norma (Cole y Chasin): 25 mm entre el gancho y el molde; parte lo pone el usuario.</t>
+          <t>ambos: la rinoscopía desde 10 min, para medir (H26, H27) completar 15</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Hoy (2026-10-22) · ver también N.º 98</t>
+          <t>Antes (regla del autor, 2026-10-16)</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -3548,7 +3654,7 @@
     <row r="36" ht="31" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>103</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -3558,22 +3664,22 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Aclimatación</t>
+          <t>Limpieza del espéculo</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Cuántos minutos espera el paciente antes de mirar o medir la nariz.</t>
+          <t>Cómo se limpia el espéculo nasal entre pacientes.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>15 min en la preparación; "desde los 10 min" en la rinoscopía</t>
+          <t>alcohol y algodón</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>ambos: la rinoscopía desde 10 min, para medir (H26, H27) completar 15</t>
+          <t>el protocolo; recuadro: instrumento semicrítico, pide desinfección de alto nivel o desechable</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -3590,7 +3696,7 @@
     <row r="37" ht="44.5" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>105</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -3600,22 +3706,22 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Limpieza del espéculo</t>
+          <t>Palpación de senos</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Cómo se limpia el espéculo nasal entre pacientes.</t>
+          <t>Si se palpan los senos paranasales en el examen.</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>alcohol y algodón</t>
+          <t>se palpan</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: instrumento semicrítico, pide desinfección de alto nivel o desechable</t>
+          <t>el protocolo; recuadro: poco valor diagnóstico por sí sola</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -3632,32 +3738,32 @@
     <row r="38" ht="31" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>115</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>H25</t>
+          <t>H26</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Palpación de senos</t>
+          <t>Valor de referencia</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Si se palpan los senos paranasales en el examen.</t>
+          <t>Resistencia nasal normal en cada fosa.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>se palpan</t>
+          <t>unilateral ≤ 0,4 Pa/(cm³/s) a 150 Pa</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: poco valor diagnóstico por sí sola</t>
+          <t>el protocolo; recuadro: Ren 2018 da 0,51 unilateral y 0,24 total en sanos; 4PR propone log Reff por percentiles</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -3674,7 +3780,7 @@
     <row r="39" ht="44.5" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>116</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -3684,22 +3790,22 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Valor de referencia</t>
+          <t>Espera tras el vasoconstrictor</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Resistencia nasal normal en cada fosa.</t>
+          <t>Cuánto se espera después del vasoconstrictor.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>unilateral ≤ 0,4 Pa/(cm³/s) a 150 Pa</t>
+          <t>15 min</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: Ren 2018 da 0,51 unilateral y 0,24 total en sanos; 4PR propone log Reff por percentiles</t>
+          <t>el protocolo; recuadro: 4PR mide a los 10 min con xilometazolina 0,1 %; el consenso pide estandarizar</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -3716,7 +3822,7 @@
     <row r="40" ht="44.5" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>117</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -3726,27 +3832,27 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Espera tras el vasoconstrictor</t>
+          <t>Resistencia que sube tras el vasoconstrictor</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Cuánto se espera después del vasoconstrictor.</t>
+          <t>Qué se informa si la nariz empeora tras el spray.</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>15 min</t>
+          <t>"efecto rebote"</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: 4PR mide a los 10 min con xilometazolina 0,1 %; el consenso pide estandarizar</t>
+          <t>Vasomotora, sin descartar un componente mecánico ("efecto rebote"), como dice el protocolo; repetir y revisar la técnica va como observación.</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Antes (regla del autor, 2026-10-16)</t>
+          <t>Hoy (2026-10-22)</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -3758,7 +3864,7 @@
     <row r="41" ht="58" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>118</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -3768,27 +3874,27 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Resistencia que sube tras el vasoconstrictor</t>
+          <t>Plazos previos</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Qué se informa si la nariz empeora tras el spray.</t>
+          <t>Qué debe cumplir el paciente antes de medir la nariz.</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>"efecto rebote"</t>
+          <t>48 h sin fármacos, 24 h sin tabaco ni alcohol, 15 min de aclimatación</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Vasomotora, sin descartar un componente mecánico ("efecto rebote"), como dice el protocolo; repetir y revisar la técnica va como observación.</t>
+          <t>el protocolo; recuadro: los plazos varían entre fuentes</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Hoy (2026-10-22)</t>
+          <t>Antes (regla del autor, 2026-10-16)</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -3800,7 +3906,7 @@
     <row r="42" ht="31" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>119</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3810,22 +3916,22 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Plazos previos</t>
+          <t>Vasoconstrictor en qué fosa</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Qué debe cumplir el paciente antes de medir la nariz.</t>
+          <t>En qué fosa se usa el vasoconstrictor.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>48 h sin fármacos, 24 h sin tabaco ni alcohol, 15 min de aclimatación</t>
+          <t>solo en la fosa que supera la referencia</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: los plazos varían entre fuentes</t>
+          <t>el protocolo (4PR descongestiona ambas en la mayoría)</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -3842,7 +3948,7 @@
     <row r="43" ht="31" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>hoy</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -3852,27 +3958,27 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Vasoconstrictor en qué fosa</t>
+          <t>Resistencia que sube con vasoconstrictor</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>En qué fosa se usa el vasoconstrictor.</t>
+          <t>En la rinomanometría, qué se informa si la nariz empeora tras el spray.</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>solo en la fosa que supera la referencia</t>
+          <t>Vasomotora, sin descartar componente mecánico (efecto rebote).</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>el protocolo (4PR descongestiona ambas en la mayoría)</t>
+          <t>Repetir la medición y revisar la técnica antes de interpretar.</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Antes (regla del autor, 2026-10-16)</t>
+          <t>Hoy (2026-10-22) · ver también N.º 117</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -3884,37 +3990,37 @@
     <row r="44" ht="44.5" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>hoy</t>
+          <t>108</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>H26</t>
+          <t>H27</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Resistencia que sube con vasoconstrictor</t>
+          <t>Repetibilidad</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>En la rinomanometría, qué se informa si la nariz empeora tras el spray.</t>
+          <t>Cuánto deben parecerse tres mediciones de la rinometría.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Vasomotora, sin descartar componente mecánico (efecto rebote).</t>
+          <t>3 registros con diferencia ≤ 0,03 en MCA1 y MCA2</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Repetir la medición y revisar la técnica antes de interpretar.</t>
+          <t>el protocolo; recuadro: límites de error probados en una fosa estándar</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Hoy (2026-10-22) · ver también N.º 117</t>
+          <t>Antes (regla del autor, 2026-10-16)</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -3926,7 +4032,7 @@
     <row r="45" ht="31" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>109</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3936,22 +4042,22 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Repetibilidad</t>
+          <t>Volúmenes</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Cuánto deben parecerse tres mediciones de la rinometría.</t>
+          <t>Cómo se definen los volúmenes de la rinometría acústica.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>3 registros con diferencia ≤ 0,03 en MCA1 y MCA2</t>
+          <t>Vol 1 narina-segundo mínimo, Vol 2 primeros 5 cm (la clase da 32 y 64 mm: no calza con el protocolo)</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: límites de error probados en una fosa estándar</t>
+          <t>el protocolo; recuadro: publicar volumen 0-5 cm (2-5 cm para mucosa) y los dos mínimos con su distancia</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3968,7 +4074,7 @@
     <row r="46" ht="44.5" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>110</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3978,22 +4084,22 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Volúmenes</t>
+          <t>Vasoconstrictor</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Cómo se definen los volúmenes de la rinometría acústica.</t>
+          <t>Cuándo se usa vasoconstrictor en la rinometría acústica.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Vol 1 narina-segundo mínimo, Vol 2 primeros 5 cm (la clase da 32 y 64 mm: no calza con el protocolo)</t>
+          <t>solo si el reposo sale fuera de rango; 2 pulverizaciones y 15 min (la clase: 2 + 2 con 5 min)</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: publicar volumen 0-5 cm (2-5 cm para mucosa) y los dos mínimos con su distancia</t>
+          <t>el protocolo; recuadro: en estudios de referencia se descongestiona a todos; estandarizar</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -4010,32 +4116,32 @@
     <row r="47" ht="44.5" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>H27</t>
+          <t>cap. 8</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Vasoconstrictor</t>
+          <t>Frecuencias de la audiometría de alta frecuencia</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Cuándo se usa vasoconstrictor en la rinometría acústica.</t>
+          <t>Qué frecuencias se miden en la audiometría de alta frecuencia.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>solo si el reposo sale fuera de rango; 2 pulverizaciones y 15 min (la clase: 2 + 2 con 5 min)</t>
+          <t>fijas: 10; 12,5; 16; 18; 19 y 20 kHz</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: en estudios de referencia se descongestiona a todos; estandarizar</t>
+          <t>el protocolo, con el "rango sensible a la ototoxicidad" en sextos de octava en el recuadro de normas</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -4052,7 +4158,7 @@
     <row r="48" ht="44.5" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -4062,22 +4168,22 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Frecuencias de la audiometría de alta frecuencia</t>
+          <t>Logoaudiometría en el monitoreo</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Qué frecuencias se miden en la audiometría de alta frecuencia.</t>
+          <t>Si en el control por ototóxicos se hace logoaudiometría.</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>fijas: 10; 12,5; 16; 18; 19 y 20 kHz</t>
+          <t>solo con indicación médica</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>el protocolo, con el "rango sensible a la ototoxicidad" en sextos de octava en el recuadro de normas</t>
+          <t>el protocolo; en el recuadro, la AAA la pide en toda base</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -4094,32 +4200,32 @@
     <row r="49" ht="31" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>48</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>cap. 8</t>
+          <t>cap. 9</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Logoaudiometría en el monitoreo</t>
+          <t>Prueba de glicerol: criterio de positivo</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Si en el control por ototóxicos se hace logoaudiometría.</t>
+          <t>Qué resultado cuenta como positivo en la prueba de glicerol.</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>solo con indicación médica</t>
+          <t>basta uno de cinco: una frecuencia ≥15 dB, logo ≥12 %, PTP ≥10 dB, menos acúfeno o menos plenitud</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; en el recuadro, la AAA la pide en toda base</t>
+          <t>el protocolo; en el recuadro, la literatura usa la mejoría de graves o de la discriminación y no los síntomas</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -4136,32 +4242,32 @@
     <row r="50" ht="44.5" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>129</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>cap. 9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Prueba de glicerol: criterio de positivo</t>
+          <t>Tasa 81,1</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Qué resultado cuenta como positivo en la prueba de glicerol.</t>
+          <t>Para qué se sube la velocidad de estímulo en el ABR del tronco.</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>basta uno de cinco: una frecuencia ≥15 dB, logo ≥12 %, PTP ≥10 dB, menos acúfeno o menos plenitud</t>
+          <t>"en sospecha de neuropatía"</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; en el recuadro, la literatura usa la mejoría de graves o de la discriminación y no los síntomas</t>
+          <t>se mantiene la tasa alta, redactada como prueba de esfuerzo de la vía (igual que H10 y #122)</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -4178,32 +4284,32 @@
     <row r="51" ht="31" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>122</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Tasa 81,1</t>
+          <t>Sospecha de neuropatía</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Para qué se sube la velocidad de estímulo en el ABR del tronco.</t>
+          <t>Qué hacer si se sospecha neuropatía auditiva en el ABR.</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>"en sospecha de neuropatía"</t>
+          <t>subir la tasa a 81,1/s</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>se mantiene la tasa alta, redactada como prueba de esfuerzo de la vía (igual que H10 y #122)</t>
+          <t>el protocolo; recuadro: lo que la define son polaridades separadas + tubo pinzado (igual que H10)</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -4220,32 +4326,32 @@
     <row r="52" ht="44.5" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>125</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Sospecha de neuropatía</t>
+          <t>Tipo de pérdida en el informe del ABR</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Qué hacer si se sospecha neuropatía auditiva en el ABR.</t>
+          <t>Si el ABR por aire basta para decir el tipo de pérdida.</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>subir la tasa a 81,1/s</t>
+          <t>concluye transmisión / SN / mixta solo con vía aérea</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: lo que la define son polaridades separadas + tubo pinzado (igual que H10)</t>
+          <t>el protocolo como sugerencia; recuadro: para clasificar hace falta ABR óseo</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -4262,32 +4368,32 @@
     <row r="53" ht="31" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>131</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Tipo de pérdida en el informe del ABR</t>
+          <t>Lactante que no duerme</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Si el ABR por aire basta para decir el tipo de pérdida.</t>
+          <t>Qué pasa si el lactante no se duerme para el examen.</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>concluye transmisión / SN / mixta solo con vía aérea</t>
+          <t>"si no duerme, el examen NO PUEDE realizarse"</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>el protocolo como sugerencia; recuadro: para clasificar hace falta ABR óseo</t>
+          <t>el protocolo; recuadro: el equipo mide el EEG y rechaza el ruido; privación de sueño solo en lactantes ambulatorios (→ cap. 17)</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -4304,32 +4410,32 @@
     <row r="54" ht="44.5" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>135</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Lactante que no duerme</t>
+          <t>Orden del examen del lactante</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Qué pasa si el lactante no se duerme para el examen.</t>
+          <t>Por qué nivel parte el ABR del lactante y cómo baja.</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>"si no duerme, el examen NO PUEDE realizarse"</t>
+          <t>parte con click a 80 dB nHL y baja de 20 en 20, sin vía ósea</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: el equipo mide el EEG y rechaza el ruido; privación de sueño solo en lactantes ambulatorios (→ cap. 17)</t>
+          <t>el protocolo; recuadro: Columbia Británica parte de 2 kHz al nivel mínimo, cambia de oído pronto y pasa a vía ósea apenas el aéreo sale elevado</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -4346,7 +4452,7 @@
     <row r="55" ht="58" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>137</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -4356,22 +4462,22 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Orden del examen del lactante</t>
+          <t>Corrección nHL → eHL</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Por qué nivel parte el ABR del lactante y cómo baja.</t>
+          <t>Cuánto se resta al nivel del ABR para estimar el umbral real.</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>parte con click a 80 dB nHL y baja de 20 en 20, sin vía ósea</t>
+          <t>LabSim: −20/−15/−10/−5 (burst 0,5-4 kHz)</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: Columbia Británica parte de 2 kHz al nivel mínimo, cambia de oído pronto y pasa a vía ósea apenas el aéreo sale elevado</t>
+          <t>la de LabSim; recuadro con la de Columbia Británica (−10/−10/−5/0)</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -4388,32 +4494,32 @@
     <row r="56" ht="31" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>139</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Corrección nHL → eHL</t>
+          <t>VEMP en la hipoacusia conductiva</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Cuánto se resta al nivel del ABR para estimar el umbral real.</t>
+          <t>Si el VEMP se puede hacer con una pérdida conductiva.</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>LabSim: −20/−15/−10/−5 (burst 0,5-4 kHz)</t>
+          <t>contraindicado, sin vibrador óseo</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>la de LabSim; recuadro con la de Columbia Británica (−10/−10/−5/0)</t>
+          <t>el protocolo; recuadro: VEMP por vía ósea como alternativa</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -4430,32 +4536,32 @@
     <row r="57" ht="31" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>141</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>VEMP en la hipoacusia conductiva</t>
+          <t>Preparación en el vértigo agudo</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Si el VEMP se puede hacer con una pérdida conductiva.</t>
+          <t>Qué se pide al paciente antes de un examen vestibular.</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>contraindicado, sin vibrador óseo</t>
+          <t>ayuno 4 h, suspender antivertiginosos 48 h</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: VEMP por vía ósea como alternativa</t>
+          <t>no aplica en el agudo: anotar qué recibió y cuándo</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -4472,32 +4578,32 @@
     <row r="58" ht="31" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>148</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Preparación en el vértigo agudo</t>
+          <t>Calórica mínima en la pérdida bilateral</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Qué se pide al paciente antes de un examen vestibular.</t>
+          <t>Cómo informar la calórica cuando fallan los dos oídos.</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>ayuno 4 h, suspender antivertiginosos 48 h</t>
+          <t>informa solo la asimetría (≥ 25 %)</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>no aplica en el agudo: anotar qué recibió y cuándo</t>
+          <t>el protocolo; recuadro: suma tibia + fría &lt; 6 °/s por oído y completar con bitérmica</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -4514,32 +4620,32 @@
     <row r="59" ht="31" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>152</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Calórica mínima en la pérdida bilateral</t>
+          <t>Posiciones de la mirada en la VNG</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Cómo informar la calórica cuando fallan los dos oídos.</t>
+          <t>Hacia dónde mira el paciente en la videonistagmografía.</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>informa solo la asimetría (≥ 25 %)</t>
+          <t>centro, derecha e izquierda (Frenzel sí pide arriba y abajo)</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: suma tibia + fría &lt; 6 °/s por oído y completar con bitérmica</t>
+          <t>el protocolo; recuadro: mirar arriba y abajo y activar el canal vertical (nistagmo hacia abajo)</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -4556,7 +4662,7 @@
     <row r="60" ht="44.5" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>154</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -4566,22 +4672,22 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Posiciones de la mirada en la VNG</t>
+          <t>Fármacos antes de la VNG</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Hacia dónde mira el paciente en la videonistagmografía.</t>
+          <t>Qué remedios se suspenden antes de la videonistagmografía.</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>centro, derecha e izquierda (Frenzel sí pide arriba y abajo)</t>
+          <t>suspender 48 h antivertiginosos, antieméticos y ansiolíticos; nada de anticonvulsivantes ni alcohol</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: mirar arriba y abajo y activar el canal vertical (nistagmo hacia abajo)</t>
+          <t>el protocolo; recuadro: anotar anticonvulsivantes y alcohol, suspender es decisión del médico</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -4598,32 +4704,32 @@
     <row r="61" ht="44.5" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>144</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Fármacos antes de la VNG</t>
+          <t>Contraindicación del VEMP aéreo</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Qué remedios se suspenden antes de la videonistagmografía.</t>
+          <t>Si el VEMP por aire se hace con pérdida conductiva o hipersensibilidad.</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>suspender 48 h antivertiginosos, antieméticos y ansiolíticos; nada de anticonvulsivantes ni alcohol</t>
+          <t>"hipoacusia de conducción" e "hipersensibilidad al sonido"</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: anotar anticonvulsivantes y alcohol, suspender es decisión del médico</t>
+          <t>se mantiene con oído medio enfermo; con gap sin oído medio que lo explique, el VEMP es la prueba que decide</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -4640,32 +4746,32 @@
     <row r="62" ht="44.5" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>156</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>28, H21</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Contraindicación del VEMP aéreo</t>
+          <t>Uno o dos audífonos</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Si el VEMP por aire se hace con pérdida conductiva o hipersensibilidad.</t>
+          <t>Si se pone un audífono o dos.</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>"hipoacusia de conducción" e "hipersensibilidad al sonido"</t>
+          <t>se adapta "el oído" y su preferencia</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>se mantiene con oído medio enfermo; con gap sin oído medio que lo explique, el VEMP es la prueba que decide</t>
+          <t>el protocolo; recuadro: dos audífonos si la pérdida es audible en ambos</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -4682,32 +4788,32 @@
     <row r="63" ht="31" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>157</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>28, H21</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Uno o dos audífonos</t>
+          <t>Control posterior</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Si se pone un audífono o dos.</t>
+          <t>Cuándo se controla al paciente después de entregar el audífono.</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>se adapta "el oído" y su preferencia</t>
+          <t>revisión visoauditiva a 1-2 años</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: dos audífonos si la pérdida es audible en ambos</t>
+          <t>el protocolo; recuadro: control presencial a las 6-12 semanas</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -4724,32 +4830,32 @@
     <row r="64" ht="31" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>159</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Control posterior</t>
+          <t>Materiales de discriminación con audífono</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Cuándo se controla al paciente después de entregar el audífono.</t>
+          <t>Con qué palabras se evalúa la discriminación con audífono.</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>revisión visoauditiva a 1-2 años</t>
+          <t>bisílabos en voz viva</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: control presencial a las 6-12 semanas</t>
+          <t>el protocolo; recuadro: los criterios de implante usan CNC/AzBio y no hay corte validado en español</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -4766,32 +4872,32 @@
     <row r="65" ht="44.5" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>161</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>31, H20</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Materiales de discriminación con audífono</t>
+          <t>Velocidad de los ejercicios de estabilización</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Con qué palabras se evalúa la discriminación con audífono.</t>
+          <t>A qué velocidad se hacen los ejercicios de mirar un punto.</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>bisílabos en voz viva</t>
+          <t>"tan rápido como se pueda mantener el blanco nítido"</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>el protocolo; recuadro: los criterios de implante usan CNC/AzBio y no hay corte validado en español</t>
+          <t>el protocolo como techo; recuadro: empezar lento</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -4808,32 +4914,32 @@
     <row r="66" ht="31" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>164</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>31, H20</t>
+          <t>32, H20</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Velocidad de los ejercicios de estabilización</t>
+          <t>Examen vestibular previo (&lt; 6 meses)</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>A qué velocidad se hacen los ejercicios de mirar un punto.</t>
+          <t>Si hay que tener un examen vestibular reciente antes de ejercitar.</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>"tan rápido como se pueda mantener el blanco nítido"</t>
+          <t>exigido antes de rehabilitar</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>el protocolo como techo; recuadro: empezar lento</t>
+          <t>Se mantiene la exigencia para rehabilitación vestibular; en un programa general de fuerza y equilibrio no se exige.</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -4850,32 +4956,32 @@
     <row r="67" ht="44.5" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>164</t>
+          <t>167</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>32, H20</t>
+          <t>36</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Examen vestibular previo (&lt; 6 meses)</t>
+          <t>"Disminución total = vasomotora"</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Si hay que tener un examen vestibular reciente antes de ejercitar.</t>
+          <t>Qué significa "vasomotora" en el informe de la nariz.</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>exigido antes de rehabilitar</t>
+          <t>rótulo del examen</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Se mantiene la exigencia para rehabilitación vestibular; en un programa general de fuerza y equilibrio no se exige.</t>
+          <t>se mantiene en el informe; recuadro: "rinitis vasomotora" es la idiopática y el término se desaconseja</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -4889,48 +4995,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="44.5" customHeight="1">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>167</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>"Disminución total = vasomotora"</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>Qué significa "vasomotora" en el informe de la nariz.</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>rótulo del examen</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>se mantiene en el informe; recuadro: "rinitis vasomotora" es la idiopática y el término se desaconseja</t>
-        </is>
-      </c>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>Antes (regla del autor, 2026-10-16)</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
-        <is>
-          <t>Resuelta: el libro sigue al protocolo</t>
-        </is>
-      </c>
-    </row>
+    <row r="68" ht="44.5" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>